<commit_message>
El calendario corre una semana
T1 del 5 al 9 de octubre, T2 del 13 al 16 (el lunes 12 es festivo), T3 del
19 al 23, T4 del 26 al 30, cierre el 2 de noviembre y aula desde el 9.
El plazo de T1 vencía antes de que el profesorado tuviera la herramienta.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Calendario_proyecto_interdisciplinar_1ESO.xlsx
+++ b/excel/Calendario_proyecto_interdisciplinar_1ESO.xlsx
@@ -4709,13 +4709,13 @@
         <v>60</v>
       </c>
       <c r="C3" s="25">
-        <v>46293.91666666667</v>
+        <v>46299.91666666667</v>
       </c>
       <c r="D3" s="25">
-        <v>46296.91666666667</v>
+        <v>46303.91666666667</v>
       </c>
       <c r="E3" s="26">
-        <v>46296.91666666667</v>
+        <v>46303.91666666667</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>61</v>
@@ -4733,13 +4733,13 @@
         <v>64</v>
       </c>
       <c r="C4" s="25">
-        <v>46299.91666666667</v>
+        <v>46307.91666666667</v>
       </c>
       <c r="D4" s="25">
-        <v>46303.91666666667</v>
+        <v>46310.91666666667</v>
       </c>
       <c r="E4" s="26">
-        <v>46303.91666666667</v>
+        <v>46310.91666666667</v>
       </c>
       <c r="F4" s="27" t="s">
         <v>65</v>
@@ -4757,13 +4757,13 @@
         <v>67</v>
       </c>
       <c r="C5" s="25">
-        <v>46307.91666666667</v>
+        <v>46313.91666666667</v>
       </c>
       <c r="D5" s="25">
-        <v>46310.91666666667</v>
+        <v>46317.91666666667</v>
       </c>
       <c r="E5" s="26">
-        <v>46310.91666666667</v>
+        <v>46317.91666666667</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>68</v>
@@ -4781,13 +4781,13 @@
         <v>70</v>
       </c>
       <c r="C6" s="25">
-        <v>46313.91666666667</v>
+        <v>46320.95833333333</v>
       </c>
       <c r="D6" s="25">
-        <v>46317.91666666667</v>
+        <v>46324.95833333333</v>
       </c>
       <c r="E6" s="26">
-        <v>46317.91666666667</v>
+        <v>46324.95833333333</v>
       </c>
       <c r="F6" s="27" t="s">
         <v>71</v>
@@ -4805,10 +4805,10 @@
         <v>73</v>
       </c>
       <c r="C7" s="28">
-        <v>46320.95833333333</v>
+        <v>46327.95833333333</v>
       </c>
       <c r="E7" s="28">
-        <v>46320.95833333333</v>
+        <v>46327.95833333333</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>

</xml_diff>

<commit_message>
Las fechas del Excel se escriben en UTC
Con medianoche local, el libro guardaba cada fecha como el día anterior:
el calendario empezaba el domingo 4 en vez del lunes 5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Calendario_proyecto_interdisciplinar_1ESO.xlsx
+++ b/excel/Calendario_proyecto_interdisciplinar_1ESO.xlsx
@@ -4709,13 +4709,13 @@
         <v>60</v>
       </c>
       <c r="C3" s="25">
-        <v>46299.91666666667</v>
+        <v>46300</v>
       </c>
       <c r="D3" s="25">
-        <v>46303.91666666667</v>
+        <v>46304</v>
       </c>
       <c r="E3" s="26">
-        <v>46303.91666666667</v>
+        <v>46304</v>
       </c>
       <c r="F3" s="27" t="s">
         <v>61</v>
@@ -4733,13 +4733,13 @@
         <v>64</v>
       </c>
       <c r="C4" s="25">
-        <v>46307.91666666667</v>
+        <v>46308</v>
       </c>
       <c r="D4" s="25">
-        <v>46310.91666666667</v>
+        <v>46311</v>
       </c>
       <c r="E4" s="26">
-        <v>46310.91666666667</v>
+        <v>46311</v>
       </c>
       <c r="F4" s="27" t="s">
         <v>65</v>
@@ -4757,13 +4757,13 @@
         <v>67</v>
       </c>
       <c r="C5" s="25">
-        <v>46313.91666666667</v>
+        <v>46314</v>
       </c>
       <c r="D5" s="25">
-        <v>46317.91666666667</v>
+        <v>46318</v>
       </c>
       <c r="E5" s="26">
-        <v>46317.91666666667</v>
+        <v>46318</v>
       </c>
       <c r="F5" s="27" t="s">
         <v>68</v>
@@ -4781,13 +4781,13 @@
         <v>70</v>
       </c>
       <c r="C6" s="25">
-        <v>46320.95833333333</v>
+        <v>46321</v>
       </c>
       <c r="D6" s="25">
-        <v>46324.95833333333</v>
+        <v>46325</v>
       </c>
       <c r="E6" s="26">
-        <v>46324.95833333333</v>
+        <v>46325</v>
       </c>
       <c r="F6" s="27" t="s">
         <v>71</v>
@@ -4805,10 +4805,10 @@
         <v>73</v>
       </c>
       <c r="C7" s="28">
-        <v>46327.95833333333</v>
+        <v>46328</v>
       </c>
       <c r="E7" s="28">
-        <v>46327.95833333333</v>
+        <v>46328</v>
       </c>
       <c r="F7" t="s">
         <v>74</v>
@@ -5553,7 +5553,7 @@
         <v>122</v>
       </c>
       <c r="Q3" s="72">
-        <v>46338.95833333333</v>
+        <v>46339</v>
       </c>
       <c r="R3" s="70" t="s">
         <v>207</v>

</xml_diff>